<commit_message>
Correctif rapprochement menages externes Hostaway
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/02_TRAVAIL/Lot10_Resultats/MASTER_CALC_Resultats.xlsx
+++ b/02_TRAVAIL/Lot10_Resultats/MASTER_CALC_Resultats.xlsx
@@ -7410,13 +7410,13 @@
         <v>2096.81</v>
       </c>
       <c r="E199" s="2" t="n">
-        <v>0</v>
+        <v>390</v>
       </c>
       <c r="F199" s="2" t="n">
-        <v>2096.81</v>
+        <v>1706.81</v>
       </c>
       <c r="G199" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -7515,13 +7515,13 @@
         <v>1640.19</v>
       </c>
       <c r="E202" s="2" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
       <c r="F202" s="2" t="n">
-        <v>1640.19</v>
+        <v>1318.19</v>
       </c>
       <c r="G202" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -7550,13 +7550,13 @@
         <v>1253.05</v>
       </c>
       <c r="E203" s="2" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="F203" s="2" t="n">
-        <v>1253.05</v>
+        <v>941.05</v>
       </c>
       <c r="G203" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -7655,13 +7655,13 @@
         <v>1129.02</v>
       </c>
       <c r="E206" s="2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F206" s="2" t="n">
-        <v>1129.02</v>
+        <v>1071.02</v>
       </c>
       <c r="G206" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -7690,13 +7690,13 @@
         <v>2073.65</v>
       </c>
       <c r="E207" s="2" t="n">
-        <v>0</v>
+        <v>440</v>
       </c>
       <c r="F207" s="2" t="n">
-        <v>2073.65</v>
+        <v>1633.65</v>
       </c>
       <c r="G207" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -7725,13 +7725,13 @@
         <v>1027.76</v>
       </c>
       <c r="E208" s="2" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="F208" s="2" t="n">
-        <v>1027.76</v>
+        <v>882.76</v>
       </c>
       <c r="G208" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -7760,13 +7760,13 @@
         <v>2123.99</v>
       </c>
       <c r="E209" s="2" t="n">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="F209" s="2" t="n">
-        <v>2123.99</v>
+        <v>1603.99</v>
       </c>
       <c r="G209" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -16195,13 +16195,13 @@
         <v>2096.81</v>
       </c>
       <c r="E450" s="2" t="n">
-        <v>0</v>
+        <v>390</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>2096.81</v>
+        <v>1706.81</v>
       </c>
       <c r="G450" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H450" s="2" t="inlineStr">
         <is>
@@ -16300,13 +16300,13 @@
         <v>1640.19</v>
       </c>
       <c r="E453" s="2" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>1640.19</v>
+        <v>1318.19</v>
       </c>
       <c r="G453" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H453" s="2" t="inlineStr">
         <is>
@@ -16335,13 +16335,13 @@
         <v>1253.05</v>
       </c>
       <c r="E454" s="2" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="F454" s="2" t="n">
-        <v>1253.05</v>
+        <v>941.05</v>
       </c>
       <c r="G454" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H454" s="2" t="inlineStr">
         <is>
@@ -16440,13 +16440,13 @@
         <v>1129.02</v>
       </c>
       <c r="E457" s="2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>1129.02</v>
+        <v>1071.02</v>
       </c>
       <c r="G457" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H457" s="2" t="inlineStr">
         <is>
@@ -16475,13 +16475,13 @@
         <v>2073.65</v>
       </c>
       <c r="E458" s="2" t="n">
-        <v>0</v>
+        <v>440</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>2073.65</v>
+        <v>1633.65</v>
       </c>
       <c r="G458" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H458" s="2" t="inlineStr">
         <is>
@@ -16510,13 +16510,13 @@
         <v>1027.76</v>
       </c>
       <c r="E459" s="2" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>1027.76</v>
+        <v>882.76</v>
       </c>
       <c r="G459" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H459" s="2" t="inlineStr">
         <is>
@@ -16545,13 +16545,13 @@
         <v>2123.99</v>
       </c>
       <c r="E460" s="2" t="n">
-        <v>0</v>
+        <v>520</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>2123.99</v>
+        <v>1603.99</v>
       </c>
       <c r="G460" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H460" s="2" t="inlineStr">
         <is>
@@ -22911,13 +22911,13 @@
         <v>2096.81</v>
       </c>
       <c r="E165" s="2" t="n">
-        <v>0</v>
+        <v>390</v>
       </c>
       <c r="F165" s="2" t="n">
-        <v>2096.81</v>
+        <v>1706.81</v>
       </c>
       <c r="G165" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="166">
@@ -22998,13 +22998,13 @@
         <v>2129.13</v>
       </c>
       <c r="E168" s="2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F168" s="2" t="n">
-        <v>2129.13</v>
+        <v>2071.13</v>
       </c>
       <c r="G168" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="169">
@@ -23027,13 +23027,13 @@
         <v>1640.19</v>
       </c>
       <c r="E169" s="2" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
       <c r="F169" s="2" t="n">
-        <v>1640.19</v>
+        <v>1318.19</v>
       </c>
       <c r="G169" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="170">
@@ -23056,13 +23056,13 @@
         <v>1253.05</v>
       </c>
       <c r="E170" s="2" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="F170" s="2" t="n">
-        <v>1253.05</v>
+        <v>941.05</v>
       </c>
       <c r="G170" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="171">
@@ -23085,13 +23085,13 @@
         <v>3316.26</v>
       </c>
       <c r="E171" s="2" t="n">
-        <v>0</v>
+        <v>440</v>
       </c>
       <c r="F171" s="2" t="n">
-        <v>3316.26</v>
+        <v>2876.26</v>
       </c>
       <c r="G171" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="172">
@@ -23114,13 +23114,13 @@
         <v>3151.75</v>
       </c>
       <c r="E172" s="2" t="n">
-        <v>0</v>
+        <v>665</v>
       </c>
       <c r="F172" s="2" t="n">
-        <v>3151.75</v>
+        <v>2486.75</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="173">
@@ -28856,13 +28856,13 @@
         <v>2096.81</v>
       </c>
       <c r="E370" s="2" t="n">
-        <v>0</v>
+        <v>390</v>
       </c>
       <c r="F370" s="2" t="n">
-        <v>2096.81</v>
+        <v>1706.81</v>
       </c>
       <c r="G370" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="371">
@@ -28943,13 +28943,13 @@
         <v>2129.13</v>
       </c>
       <c r="E373" s="2" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F373" s="2" t="n">
-        <v>2129.13</v>
+        <v>2071.13</v>
       </c>
       <c r="G373" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="374">
@@ -28972,13 +28972,13 @@
         <v>1640.19</v>
       </c>
       <c r="E374" s="2" t="n">
-        <v>0</v>
+        <v>322</v>
       </c>
       <c r="F374" s="2" t="n">
-        <v>1640.19</v>
+        <v>1318.19</v>
       </c>
       <c r="G374" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="375">
@@ -29001,13 +29001,13 @@
         <v>1253.05</v>
       </c>
       <c r="E375" s="2" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="F375" s="2" t="n">
-        <v>1253.05</v>
+        <v>941.05</v>
       </c>
       <c r="G375" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="376">
@@ -29030,13 +29030,13 @@
         <v>3316.26</v>
       </c>
       <c r="E376" s="2" t="n">
-        <v>0</v>
+        <v>440</v>
       </c>
       <c r="F376" s="2" t="n">
-        <v>3316.26</v>
+        <v>2876.26</v>
       </c>
       <c r="G376" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="377">
@@ -29059,13 +29059,13 @@
         <v>3151.75</v>
       </c>
       <c r="E377" s="2" t="n">
-        <v>0</v>
+        <v>665</v>
       </c>
       <c r="F377" s="2" t="n">
-        <v>3151.75</v>
+        <v>2486.75</v>
       </c>
       <c r="G377" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="378">
@@ -30112,10 +30112,10 @@
         <v>286053.08</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>267.09</v>
+        <v>2454.09</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>285785.99</v>
+        <v>283598.99</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -30133,10 +30133,10 @@
         <v>283709.6</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>267.09</v>
+        <v>2454.09</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>283442.51</v>
+        <v>281255.51</v>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Standard menage analytique HC (TYPE_FLUX_019) + ecart (018) - net = cout complet
</commit_message>
<xml_diff>
--- a/02_TRAVAIL/Lot10_Resultats/MASTER_CALC_Resultats.xlsx
+++ b/02_TRAVAIL/Lot10_Resultats/MASTER_CALC_Resultats.xlsx
@@ -434,14 +434,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I527"/>
+  <dimension ref="A1:I532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
@@ -7375,13 +7375,13 @@
         <v>1378.1</v>
       </c>
       <c r="E198" s="2" t="n">
-        <v>151.33</v>
+        <v>412.33</v>
       </c>
       <c r="F198" s="2" t="n">
-        <v>1226.77</v>
+        <v>965.77</v>
       </c>
       <c r="G198" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
@@ -7410,13 +7410,13 @@
         <v>2120.81</v>
       </c>
       <c r="E199" s="2" t="n">
-        <v>390</v>
+        <v>804</v>
       </c>
       <c r="F199" s="2" t="n">
-        <v>1730.81</v>
+        <v>1316.81</v>
       </c>
       <c r="G199" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
@@ -7480,13 +7480,13 @@
         <v>1000.11</v>
       </c>
       <c r="E201" s="2" t="n">
-        <v>81.84999999999999</v>
+        <v>226.85</v>
       </c>
       <c r="F201" s="2" t="n">
-        <v>918.26</v>
+        <v>773.26</v>
       </c>
       <c r="G201" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H201" s="2" t="inlineStr">
         <is>
@@ -7515,13 +7515,13 @@
         <v>1640.19</v>
       </c>
       <c r="E202" s="2" t="n">
-        <v>325</v>
+        <v>644</v>
       </c>
       <c r="F202" s="2" t="n">
-        <v>1315.19</v>
+        <v>996.1900000000001</v>
       </c>
       <c r="G202" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
@@ -7550,13 +7550,13 @@
         <v>1253.05</v>
       </c>
       <c r="E203" s="2" t="n">
-        <v>312</v>
+        <v>624</v>
       </c>
       <c r="F203" s="2" t="n">
-        <v>941.05</v>
+        <v>629.05</v>
       </c>
       <c r="G203" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
@@ -7585,13 +7585,13 @@
         <v>2139.75</v>
       </c>
       <c r="E204" s="2" t="n">
-        <v>0</v>
+        <v>275</v>
       </c>
       <c r="F204" s="2" t="n">
-        <v>2139.75</v>
+        <v>1864.75</v>
       </c>
       <c r="G204" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
@@ -7620,13 +7620,13 @@
         <v>2343.48</v>
       </c>
       <c r="E205" s="2" t="n">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="F205" s="2" t="n">
-        <v>2288.48</v>
+        <v>2233.48</v>
       </c>
       <c r="G205" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
@@ -7655,13 +7655,13 @@
         <v>1129.02</v>
       </c>
       <c r="E206" s="2" t="n">
-        <v>58</v>
+        <v>116</v>
       </c>
       <c r="F206" s="2" t="n">
-        <v>1071.02</v>
+        <v>1013.02</v>
       </c>
       <c r="G206" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
@@ -7690,13 +7690,13 @@
         <v>2073.65</v>
       </c>
       <c r="E207" s="2" t="n">
-        <v>440</v>
+        <v>880</v>
       </c>
       <c r="F207" s="2" t="n">
-        <v>1633.65</v>
+        <v>1193.65</v>
       </c>
       <c r="G207" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
@@ -7725,13 +7725,13 @@
         <v>1027.76</v>
       </c>
       <c r="E208" s="2" t="n">
-        <v>145</v>
+        <v>290</v>
       </c>
       <c r="F208" s="2" t="n">
-        <v>882.76</v>
+        <v>737.76</v>
       </c>
       <c r="G208" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
@@ -7760,13 +7760,13 @@
         <v>2153.99</v>
       </c>
       <c r="E209" s="2" t="n">
-        <v>520</v>
+        <v>1070</v>
       </c>
       <c r="F209" s="2" t="n">
-        <v>1633.99</v>
+        <v>1083.99</v>
       </c>
       <c r="G209" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
@@ -7795,13 +7795,13 @@
         <v>1400.05</v>
       </c>
       <c r="E210" s="2" t="n">
-        <v>62.33</v>
+        <v>352.33</v>
       </c>
       <c r="F210" s="2" t="n">
-        <v>1337.72</v>
+        <v>1047.72</v>
       </c>
       <c r="G210" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
@@ -7830,13 +7830,13 @@
         <v>467.89</v>
       </c>
       <c r="E211" s="2" t="n">
-        <v>39.48</v>
+        <v>155.48</v>
       </c>
       <c r="F211" s="2" t="n">
-        <v>428.41</v>
+        <v>312.41</v>
       </c>
       <c r="G211" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H211" s="2" t="inlineStr">
         <is>
@@ -7865,13 +7865,13 @@
         <v>374.44</v>
       </c>
       <c r="E212" s="2" t="n">
-        <v>110</v>
+        <v>220</v>
       </c>
       <c r="F212" s="2" t="n">
-        <v>264.44</v>
+        <v>154.44</v>
       </c>
       <c r="G212" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
@@ -18670,13 +18670,13 @@
         <v>0</v>
       </c>
       <c r="E519" s="2" t="n">
-        <v>151.33</v>
+        <v>412.33</v>
       </c>
       <c r="F519" s="2" t="n">
-        <v>-151.33</v>
+        <v>-412.33</v>
       </c>
       <c r="G519" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H519" s="2" t="inlineStr">
         <is>
@@ -18709,13 +18709,13 @@
         <v>24</v>
       </c>
       <c r="E520" s="2" t="n">
-        <v>0</v>
+        <v>414</v>
       </c>
       <c r="F520" s="2" t="n">
-        <v>24</v>
+        <v>-390</v>
       </c>
       <c r="G520" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H520" s="2" t="inlineStr">
         <is>
@@ -18748,13 +18748,13 @@
         <v>0</v>
       </c>
       <c r="E521" s="2" t="n">
-        <v>81.84999999999999</v>
+        <v>226.85</v>
       </c>
       <c r="F521" s="2" t="n">
-        <v>-81.84999999999999</v>
+        <v>-226.85</v>
       </c>
       <c r="G521" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H521" s="2" t="inlineStr">
         <is>
@@ -18787,13 +18787,13 @@
         <v>0</v>
       </c>
       <c r="E522" s="2" t="n">
+        <v>322</v>
+      </c>
+      <c r="F522" s="2" t="n">
+        <v>-322</v>
+      </c>
+      <c r="G522" s="2" t="n">
         <v>3</v>
-      </c>
-      <c r="F522" s="2" t="n">
-        <v>-3</v>
-      </c>
-      <c r="G522" s="2" t="n">
-        <v>1</v>
       </c>
       <c r="H522" s="2" t="inlineStr">
         <is>
@@ -18814,25 +18814,25 @@
       </c>
       <c r="B523" s="2" t="inlineStr">
         <is>
-          <t>LOG_0008</t>
+          <t>LOG_0007</t>
         </is>
       </c>
       <c r="C523" s="2" t="inlineStr">
         <is>
-          <t>PROP_0008</t>
+          <t>PROP_0007</t>
         </is>
       </c>
       <c r="D523" s="2" t="n">
-        <v>897.14</v>
+        <v>0</v>
       </c>
       <c r="E523" s="2" t="n">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="F523" s="2" t="n">
-        <v>897.14</v>
+        <v>-312</v>
       </c>
       <c r="G523" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H523" s="2" t="inlineStr">
         <is>
@@ -18853,25 +18853,25 @@
       </c>
       <c r="B524" s="2" t="inlineStr">
         <is>
-          <t>LOG_0009</t>
+          <t>LOG_0008</t>
         </is>
       </c>
       <c r="C524" s="2" t="inlineStr">
         <is>
-          <t>PROP_0003</t>
+          <t>PROP_0008</t>
         </is>
       </c>
       <c r="D524" s="2" t="n">
-        <v>2343.48</v>
+        <v>897.14</v>
       </c>
       <c r="E524" s="2" t="n">
-        <v>0</v>
+        <v>275</v>
       </c>
       <c r="F524" s="2" t="n">
-        <v>2343.48</v>
+        <v>622.14</v>
       </c>
       <c r="G524" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H524" s="2" t="inlineStr">
         <is>
@@ -18892,25 +18892,25 @@
       </c>
       <c r="B525" s="2" t="inlineStr">
         <is>
-          <t>LOG_0013</t>
+          <t>LOG_0009</t>
         </is>
       </c>
       <c r="C525" s="2" t="inlineStr">
         <is>
-          <t>PROP_0009</t>
+          <t>PROP_0003</t>
         </is>
       </c>
       <c r="D525" s="2" t="n">
-        <v>30</v>
+        <v>2343.48</v>
       </c>
       <c r="E525" s="2" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="F525" s="2" t="n">
-        <v>30</v>
+        <v>2288.48</v>
       </c>
       <c r="G525" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H525" s="2" t="inlineStr">
         <is>
@@ -18931,22 +18931,22 @@
       </c>
       <c r="B526" s="2" t="inlineStr">
         <is>
-          <t>LOG_0014</t>
+          <t>LOG_0010</t>
         </is>
       </c>
       <c r="C526" s="2" t="inlineStr">
         <is>
-          <t>PROP_0010</t>
+          <t>PROP_0005</t>
         </is>
       </c>
       <c r="D526" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E526" s="2" t="n">
-        <v>33.33</v>
+        <v>58</v>
       </c>
       <c r="F526" s="2" t="n">
-        <v>-33.33</v>
+        <v>-58</v>
       </c>
       <c r="G526" s="2" t="n">
         <v>1</v>
@@ -18970,22 +18970,22 @@
       </c>
       <c r="B527" s="2" t="inlineStr">
         <is>
-          <t>LOG_0015</t>
+          <t>LOG_0011</t>
         </is>
       </c>
       <c r="C527" s="2" t="inlineStr">
         <is>
-          <t>PROP_0011</t>
+          <t>PROP_0008</t>
         </is>
       </c>
       <c r="D527" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E527" s="2" t="n">
-        <v>39.48</v>
+        <v>440</v>
       </c>
       <c r="F527" s="2" t="n">
-        <v>-39.48</v>
+        <v>-440</v>
       </c>
       <c r="G527" s="2" t="n">
         <v>1</v>
@@ -18996,6 +18996,201 @@
         </is>
       </c>
       <c r="I527" s="2" t="inlineStr">
+        <is>
+          <t>Flux HC presents</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>LOG_0012</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>PROP_0009</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E528" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="F528" s="2" t="n">
+        <v>-145</v>
+      </c>
+      <c r="G528" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H528" s="2" t="inlineStr">
+        <is>
+          <t>HORS_COMPTA</t>
+        </is>
+      </c>
+      <c r="I528" s="2" t="inlineStr">
+        <is>
+          <t>Flux HC presents</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B529" s="2" t="inlineStr">
+        <is>
+          <t>LOG_0013</t>
+        </is>
+      </c>
+      <c r="C529" s="2" t="inlineStr">
+        <is>
+          <t>PROP_0009</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E529" s="2" t="n">
+        <v>550</v>
+      </c>
+      <c r="F529" s="2" t="n">
+        <v>-520</v>
+      </c>
+      <c r="G529" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H529" s="2" t="inlineStr">
+        <is>
+          <t>HORS_COMPTA</t>
+        </is>
+      </c>
+      <c r="I529" s="2" t="inlineStr">
+        <is>
+          <t>Flux HC presents</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B530" s="2" t="inlineStr">
+        <is>
+          <t>LOG_0014</t>
+        </is>
+      </c>
+      <c r="C530" s="2" t="inlineStr">
+        <is>
+          <t>PROP_0010</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E530" s="2" t="n">
+        <v>323.33</v>
+      </c>
+      <c r="F530" s="2" t="n">
+        <v>-323.33</v>
+      </c>
+      <c r="G530" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H530" s="2" t="inlineStr">
+        <is>
+          <t>HORS_COMPTA</t>
+        </is>
+      </c>
+      <c r="I530" s="2" t="inlineStr">
+        <is>
+          <t>Flux HC presents</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B531" s="2" t="inlineStr">
+        <is>
+          <t>LOG_0015</t>
+        </is>
+      </c>
+      <c r="C531" s="2" t="inlineStr">
+        <is>
+          <t>PROP_0011</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E531" s="2" t="n">
+        <v>155.48</v>
+      </c>
+      <c r="F531" s="2" t="n">
+        <v>-155.48</v>
+      </c>
+      <c r="G531" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H531" s="2" t="inlineStr">
+        <is>
+          <t>HORS_COMPTA</t>
+        </is>
+      </c>
+      <c r="I531" s="2" t="inlineStr">
+        <is>
+          <t>Flux HC presents</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B532" s="2" t="inlineStr">
+        <is>
+          <t>LOG_0016</t>
+        </is>
+      </c>
+      <c r="C532" s="2" t="inlineStr">
+        <is>
+          <t>PROP_0012</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E532" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="F532" s="2" t="n">
+        <v>-110</v>
+      </c>
+      <c r="G532" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H532" s="2" t="inlineStr">
+        <is>
+          <t>HORS_COMPTA</t>
+        </is>
+      </c>
+      <c r="I532" s="2" t="inlineStr">
         <is>
           <t>Flux HC presents</t>
         </is>
@@ -19019,7 +19214,7 @@
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
   </cols>
@@ -23779,13 +23974,13 @@
         <v>1378.1</v>
       </c>
       <c r="E164" s="2" t="n">
-        <v>151.33</v>
+        <v>412.33</v>
       </c>
       <c r="F164" s="2" t="n">
-        <v>1226.77</v>
+        <v>965.77</v>
       </c>
       <c r="G164" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="165">
@@ -23808,13 +24003,13 @@
         <v>2120.81</v>
       </c>
       <c r="E165" s="2" t="n">
-        <v>390</v>
+        <v>804</v>
       </c>
       <c r="F165" s="2" t="n">
-        <v>1730.81</v>
+        <v>1316.81</v>
       </c>
       <c r="G165" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="166">
@@ -23837,13 +24032,13 @@
         <v>2343.48</v>
       </c>
       <c r="E166" s="2" t="n">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="F166" s="2" t="n">
-        <v>2288.48</v>
+        <v>2233.48</v>
       </c>
       <c r="G166" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="167">
@@ -23895,13 +24090,13 @@
         <v>2129.13</v>
       </c>
       <c r="E168" s="2" t="n">
-        <v>139.85</v>
+        <v>342.85</v>
       </c>
       <c r="F168" s="2" t="n">
-        <v>1989.28</v>
+        <v>1786.28</v>
       </c>
       <c r="G168" s="2" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="169">
@@ -23924,13 +24119,13 @@
         <v>1640.19</v>
       </c>
       <c r="E169" s="2" t="n">
-        <v>325</v>
+        <v>644</v>
       </c>
       <c r="F169" s="2" t="n">
-        <v>1315.19</v>
+        <v>996.1900000000001</v>
       </c>
       <c r="G169" s="2" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="170">
@@ -23953,13 +24148,13 @@
         <v>1253.05</v>
       </c>
       <c r="E170" s="2" t="n">
-        <v>312</v>
+        <v>624</v>
       </c>
       <c r="F170" s="2" t="n">
-        <v>941.05</v>
+        <v>629.05</v>
       </c>
       <c r="G170" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="171">
@@ -23982,13 +24177,13 @@
         <v>4213.4</v>
       </c>
       <c r="E171" s="2" t="n">
-        <v>440</v>
+        <v>1155</v>
       </c>
       <c r="F171" s="2" t="n">
-        <v>3773.4</v>
+        <v>3058.4</v>
       </c>
       <c r="G171" s="2" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="172">
@@ -24011,13 +24206,13 @@
         <v>3181.75</v>
       </c>
       <c r="E172" s="2" t="n">
-        <v>665</v>
+        <v>1360</v>
       </c>
       <c r="F172" s="2" t="n">
-        <v>2516.75</v>
+        <v>1821.75</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="173">
@@ -24040,13 +24235,13 @@
         <v>1400.05</v>
       </c>
       <c r="E173" s="2" t="n">
-        <v>62.33</v>
+        <v>352.33</v>
       </c>
       <c r="F173" s="2" t="n">
-        <v>1337.72</v>
+        <v>1047.72</v>
       </c>
       <c r="G173" s="2" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="174">
@@ -24069,13 +24264,13 @@
         <v>467.89</v>
       </c>
       <c r="E174" s="2" t="n">
-        <v>39.48</v>
+        <v>155.48</v>
       </c>
       <c r="F174" s="2" t="n">
-        <v>428.41</v>
+        <v>312.41</v>
       </c>
       <c r="G174" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="175">
@@ -24098,13 +24293,13 @@
         <v>374.44</v>
       </c>
       <c r="E175" s="2" t="n">
-        <v>110</v>
+        <v>220</v>
       </c>
       <c r="F175" s="2" t="n">
-        <v>264.44</v>
+        <v>154.44</v>
       </c>
       <c r="G175" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="176">
@@ -31009,10 +31204,10 @@
         <v>298032.75</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2763.08</v>
+        <v>6253.08</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>295269.67</v>
+        <v>291779.67</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
@@ -31051,10 +31246,10 @@
         <v>14323.15</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>308.99</v>
+        <v>3798.99</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>14014.16</v>
+        <v>10524.16</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>

</xml_diff>